<commit_message>
Add Club Sources tab and Apps Script auto-updater
- New 'Club Sources' tab seeded with 12 Vancouver clubs; drives automation
- apps_script/BasketballUpdater.gs: reads Club Sources, fetches each club's
  public site on a daily trigger, appends dated tryout/camp candidates
  flagged REVIEW with de-duping

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NFJDfPdQrdUX4za1wFnqHF
</commit_message>
<xml_diff>
--- a/basketball_club_updates.xlsx
+++ b/basketball_club_updates.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Club Tryouts" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Club Camps" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Lists" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Club Sources" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -69,7 +70,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +85,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -133,6 +139,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2470,4 +2479,316 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Club Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The Apps Script updater reads this tab. Fill in each club's website / registration page and the script pulls tryout &amp; camp dates from it on a schedule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Club / Program</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Website URL</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Registration / Linktree URL</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Auto-pull? (Y/N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Split Second Basketball</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr"/>
+      <c r="C5" s="11" t="inlineStr"/>
+      <c r="D5" s="11" t="inlineStr"/>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Rain City</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr"/>
+      <c r="C6" s="11" t="inlineStr"/>
+      <c r="D6" s="11" t="inlineStr"/>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Vancity</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr"/>
+      <c r="C7" s="11" t="inlineStr"/>
+      <c r="D7" s="11" t="inlineStr"/>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Greenlight</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr"/>
+      <c r="C8" s="11" t="inlineStr"/>
+      <c r="D8" s="11" t="inlineStr"/>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Journey</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr"/>
+      <c r="C9" s="11" t="inlineStr"/>
+      <c r="D9" s="11" t="inlineStr"/>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Squad International</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr"/>
+      <c r="C10" s="11" t="inlineStr"/>
+      <c r="D10" s="11" t="inlineStr"/>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr"/>
+      <c r="C11" s="11" t="inlineStr"/>
+      <c r="D11" s="11" t="inlineStr"/>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Alamat Allstars</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr"/>
+      <c r="C12" s="11" t="inlineStr"/>
+      <c r="D12" s="11" t="inlineStr"/>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Prospect Basketball</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr"/>
+      <c r="C13" s="11" t="inlineStr"/>
+      <c r="D13" s="11" t="inlineStr"/>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>RBL Basketball</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr"/>
+      <c r="C14" s="11" t="inlineStr"/>
+      <c r="D14" s="11" t="inlineStr"/>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Dime Hoops Basketball</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr"/>
+      <c r="C15" s="11" t="inlineStr"/>
+      <c r="D15" s="11" t="inlineStr"/>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Empower Basketball</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr"/>
+      <c r="C16" s="11" t="inlineStr"/>
+      <c r="D16" s="11" t="inlineStr"/>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Populate workbook with researched Vancouver club data
- Club Sources tab: confirmed website/registration/Instagram URLs for 11 of
  12 clubs (Alamat Allstars not found online; Prospect is IG/FB-only)
- Club Tryouts / Club Camps seeded with real leads; search-derived dates
  flagged REVIEW, Journey's Aug 17-21 2026 camp confirmed via venue page

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NFJDfPdQrdUX4za1wFnqHF
</commit_message>
<xml_diff>
--- a/basketball_club_updates.xlsx
+++ b/basketball_club_updates.xlsx
@@ -760,7 +760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -907,46 +907,160 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n"/>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="8" t="n"/>
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Rain City</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>U10-U18 B/G</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>RayCam Co-op Community Centre</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>https://www.raincitybasketball.ca/register</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>ID sessions $30. Dates shown are the Spring season window (Mar 30-Jun 15); confirm exact tryout date/time on site.</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n"/>
-      <c r="B6" s="9" t="n"/>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="n"/>
-      <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
-      <c r="L6" s="9" t="n"/>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Boys 9-17</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr"/>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>https://drivebasketball.com/drive-team-tryouts/</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>Fall club tryouts ~Sept 9 (year unconfirmed); registration opens mid-July. Confirm on site.</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Squad International</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Grades 3-7</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr"/>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>St Patrick's HS gym</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr"/>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>https://squadbasketball.hoopstir.com/</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>'Dream Hoops Combine' selects teams. A Sept 7-8 combine date appears in search but likely 2024 - confirm 2026 date on Hoopstir portal.</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n"/>
@@ -1423,34 +1537,6 @@
       <c r="J41" s="8" t="n"/>
       <c r="K41" s="8" t="n"/>
       <c r="L41" s="8" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="9" t="n"/>
-      <c r="B42" s="9" t="n"/>
-      <c r="C42" s="9" t="n"/>
-      <c r="D42" s="9" t="n"/>
-      <c r="E42" s="9" t="n"/>
-      <c r="F42" s="9" t="n"/>
-      <c r="G42" s="9" t="n"/>
-      <c r="H42" s="9" t="n"/>
-      <c r="I42" s="9" t="n"/>
-      <c r="J42" s="9" t="n"/>
-      <c r="K42" s="9" t="n"/>
-      <c r="L42" s="9" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="n"/>
-      <c r="B43" s="8" t="n"/>
-      <c r="C43" s="8" t="n"/>
-      <c r="D43" s="8" t="n"/>
-      <c r="E43" s="8" t="n"/>
-      <c r="F43" s="8" t="n"/>
-      <c r="G43" s="8" t="n"/>
-      <c r="H43" s="8" t="n"/>
-      <c r="I43" s="8" t="n"/>
-      <c r="J43" s="8" t="n"/>
-      <c r="K43" s="8" t="n"/>
-      <c r="L43" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1474,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1643,68 +1729,246 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n"/>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="8" t="n"/>
-      <c r="M5" s="8" t="n"/>
-      <c r="N5" s="8" t="n"/>
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Journey</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Journey Basketball Camp</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Day Camp</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Ages 6-8</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Champlain Heights Community Centre</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr"/>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>https://champlainheightscc.ca/event/journey-basketball-camp-6-8yrs-3/</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>Mon-Fri 1:00-2:30 PM. Confirmed via community-centre event page; verify cost.</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n"/>
-      <c r="B6" s="9" t="n"/>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="n"/>
-      <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
-      <c r="L6" s="9" t="n"/>
-      <c r="M6" s="9" t="n"/>
-      <c r="N6" s="9" t="n"/>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>HoopSoles Rising Stars Camp</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Day Camp</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Ages 8-16</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>The Hoop Vancouver</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>https://drivebasketball.com/camps/</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>July camps ~$1000+tax, Aug ~$800+tax (unverified search snippet). Confirm dates on site.</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
-      <c r="M7" s="8" t="n"/>
-      <c r="N7" s="8" t="n"/>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Greenlight</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Foundations Camp</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Skills Camp</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr"/>
+      <c r="E7" s="8" t="inlineStr"/>
+      <c r="F7" s="8" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Killarney Community Centre</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr"/>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>https://ca.apm.activecommunities.com/vancouver/Activity_Search/greenlight-basketball---foundations-camp/521010</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>Dates/cost not public in search; confirm on Vancouver ActiveNet listing.</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="n"/>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
-      <c r="J8" s="9" t="n"/>
-      <c r="K8" s="9" t="n"/>
-      <c r="L8" s="9" t="n"/>
-      <c r="M8" s="9" t="n"/>
-      <c r="N8" s="9" t="n"/>
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Split Second</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>3-on-3 Summer League</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Clinic</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Grades 4-12</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr"/>
+      <c r="J8" s="9" t="inlineStr"/>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>https://splitsecondbasketball.leagueapps.com/</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>Summer league (Tue/Thu). Confirm session dates on LeagueApps.</t>
+        </is>
+      </c>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n"/>
@@ -2249,22 +2513,6 @@
       <c r="L42" s="9" t="n"/>
       <c r="M42" s="9" t="n"/>
       <c r="N42" s="9" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="n"/>
-      <c r="B43" s="8" t="n"/>
-      <c r="C43" s="8" t="n"/>
-      <c r="D43" s="8" t="n"/>
-      <c r="E43" s="8" t="n"/>
-      <c r="F43" s="8" t="n"/>
-      <c r="G43" s="8" t="n"/>
-      <c r="H43" s="8" t="n"/>
-      <c r="I43" s="8" t="n"/>
-      <c r="J43" s="8" t="n"/>
-      <c r="K43" s="8" t="n"/>
-      <c r="L43" s="8" t="n"/>
-      <c r="M43" s="8" t="n"/>
-      <c r="N43" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2550,9 +2798,21 @@
           <t>Split Second Basketball</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>https://www.splitsecondbasketball.com/</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>https://splitsecondbasketball.leagueapps.com/</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/splitsecondbasketball/</t>
+        </is>
+      </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Vancouver</t>
@@ -2570,9 +2830,21 @@
           <t>Rain City</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>https://www.raincitybasketball.ca/</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>https://www.raincitybasketball.ca/register</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/raincitybasketball/</t>
+        </is>
+      </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Vancouver</t>
@@ -2590,12 +2862,24 @@
           <t>Vancity</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>https://vancitybasketball.com/</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>https://vancitybasketball.teamsportsadmin.com/events</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vancitybasketballacademy/</t>
+        </is>
+      </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>North Vancouver</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
@@ -2610,9 +2894,17 @@
           <t>Greenlight</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr"/>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>https://www.greenlightbasketball.ca/</t>
+        </is>
+      </c>
       <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/greenlightbball/</t>
+        </is>
+      </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Vancouver</t>
@@ -2630,9 +2922,21 @@
           <t>Journey</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.journeybasketball.ca/</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.journeybasketball.ca/development-programs</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/journey_basketball/</t>
+        </is>
+      </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
           <t>Vancouver</t>
@@ -2650,9 +2954,21 @@
           <t>Squad International</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>https://www.squadbasketball.net/</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>https://squadbasketball.hoopstir.com/</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/international_squad/</t>
+        </is>
+      </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Vancouver</t>
@@ -2670,12 +2986,20 @@
           <t>Drive</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>https://drivebasketball.com/</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>https://drivebasketball.com/camps/</t>
+        </is>
+      </c>
       <c r="D11" s="11" t="inlineStr"/>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Surrey / Vancouver</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
@@ -2700,7 +3024,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2711,8 +3035,16 @@
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/Prospectsbasketballacademy/</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/prospectsbasketballbc/</t>
+        </is>
+      </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Vancouver</t>
@@ -2720,7 +3052,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -2730,9 +3062,21 @@
           <t>RBL Basketball</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>https://rblbasketball.com/</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>https://rblbasketball.com/skill-development/</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/rblbasketball/</t>
+        </is>
+      </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Vancouver</t>
@@ -2750,12 +3094,24 @@
           <t>Dime Hoops Basketball</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>https://dimehoops.ca/</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>https://www.dimehoops.ca/registration</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/dimehoopsbc/</t>
+        </is>
+      </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -2770,12 +3126,24 @@
           <t>Empower Basketball</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr"/>
-      <c r="C16" s="11" t="inlineStr"/>
-      <c r="D16" s="11" t="inlineStr"/>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>https://www.empowerbasketball.ca/</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>https://www.empowerbasketball.ca/programs-and-locations</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/empowerbclub/</t>
+        </is>
+      </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">

</xml_diff>